<commit_message>
Publish 2026-10-30 06:28 UTC (src 5a73374)
</commit_message>
<xml_diff>
--- a/Data/Farmer_Recourse.xlsx
+++ b/Data/Farmer_Recourse.xlsx
@@ -329,17 +329,17 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wheat T/acre</t>
+          <t xml:space="preserve">Wheat tons/acre</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Corn T/acre</t>
+          <t xml:space="preserve">Corn tons/acre</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beets T/acre</t>
+          <t xml:space="preserve">Beets tons/acre</t>
         </is>
       </c>
     </row>
@@ -365,32 +365,32 @@
     <row r="10">
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sell wheat (T)</t>
+          <t xml:space="preserve">Sell wheat (tons)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sell corn (T)</t>
+          <t xml:space="preserve">Sell corn (tons)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sell beets at quota price (T)</t>
+          <t xml:space="preserve">Sell beets at quota price (tons)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sell beets above quota (T)</t>
+          <t xml:space="preserve">Sell beets above quota (tons)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Buy wheat (T)</t>
+          <t xml:space="preserve">Buy wheat (tons)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Buy corn (T)</t>
+          <t xml:space="preserve">Buy corn (tons)</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -431,7 +431,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Price ($/T); purchases negative</t>
+          <t xml:space="preserve">Price ($/ton); purchases negative</t>
         </is>
       </c>
       <c r="B12" s="4">
@@ -696,17 +696,17 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wheat T/acre</t>
+          <t xml:space="preserve">Wheat tons/acre</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Corn T/acre</t>
+          <t xml:space="preserve">Corn tons/acre</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beets T/acre</t>
+          <t xml:space="preserve">Beets tons/acre</t>
         </is>
       </c>
     </row>
@@ -770,32 +770,32 @@
     <row r="12">
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sell wheat (T)</t>
+          <t xml:space="preserve">Sell wheat (tons)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sell corn (T)</t>
+          <t xml:space="preserve">Sell corn (tons)</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sell beets at quota price (T)</t>
+          <t xml:space="preserve">Sell beets at quota price (tons)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sell beets above quota (T)</t>
+          <t xml:space="preserve">Sell beets above quota (tons)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Buy wheat (T)</t>
+          <t xml:space="preserve">Buy wheat (tons)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Buy corn (T)</t>
+          <t xml:space="preserve">Buy corn (tons)</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -894,7 +894,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Price ($/T); purchases negative</t>
+          <t xml:space="preserve">Price ($/ton); purchases negative</t>
         </is>
       </c>
       <c r="B16" s="4">
@@ -1154,7 +1154,7 @@
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Type 120, 80, 300 in B5:D5, remove B5:D5 from the changing cells and re-solve: the mean plan earns $107,240.</t>
+          <t xml:space="preserve">Type 120, 80, 300 in B5:D5, remove B5:D5 from the changing cells and re-solve: the mean plan's expected profit.</t>
         </is>
       </c>
     </row>

</xml_diff>